<commit_message>
modified missing records related to birth data set 2000
</commit_message>
<xml_diff>
--- a/notebooks/2000_Birth/01_missing_values.xlsx
+++ b/notebooks/2000_Birth/01_missing_values.xlsx
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>701047</v>
+        <v>221</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -525,7 +525,7 @@
         <v>347528</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>33.1</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>700917</v>
+        <v>91</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -552,51 +552,51 @@
         <v>347658</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Birh_Year_2.0</t>
+          <t>Registered_District</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>347749</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Birh_Year</t>
+          <t>Birh_Year_2.0</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -606,7 +606,7 @@
         <v>347749</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -616,14 +616,14 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -633,7 +633,7 @@
         <v>347749</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -643,10 +643,10 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -660,61 +660,61 @@
         <v>347749</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Birth_Order 2.0</t>
+          <t>Birth_Month</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>347749</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Birth_Month</t>
+          <t>Birh_Year</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>347749</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -724,10 +724,10 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         <v>347749</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -768,34 +768,34 @@
         <v>347749</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Marital_Status</t>
+          <t>Birth_Order 2.0</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>347749</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -805,14 +805,14 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>700826</v>
+        <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>66.8</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -822,13 +822,13 @@
         <v>347749</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>33.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Registered_District</t>
+          <t>Marital_Status</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -843,10 +843,10 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1048575</v>
+        <v>347749</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>100</v>
@@ -873,7 +873,7 @@
         <v>26</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1048575</v>
+        <v>347749</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>100</v>
@@ -894,7 +894,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1048575</v>
+        <v>347749</v>
       </c>
     </row>
     <row r="3">
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>8410224</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6">
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>57.29</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
creating complete data files 2000
</commit_message>
<xml_diff>
--- a/notebooks/2000_Birth/01_missing_values.xlsx
+++ b/notebooks/2000_Birth/01_missing_values.xlsx
@@ -522,7 +522,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>347528</v>
+        <v>347517</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>99.90000000000001</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0</v>
@@ -549,7 +549,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>347658</v>
+        <v>347650</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>100</v>
@@ -576,7 +576,7 @@
         <v>25</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>100</v>
@@ -603,7 +603,7 @@
         <v>57</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>100</v>
@@ -630,7 +630,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>100</v>
@@ -657,7 +657,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>100</v>
@@ -684,7 +684,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -711,7 +711,7 @@
         <v>57</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -738,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>100</v>
@@ -765,7 +765,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>100</v>
@@ -792,7 +792,7 @@
         <v>14</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>100</v>
@@ -819,7 +819,7 @@
         <v>43</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>100</v>
@@ -846,7 +846,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>100</v>
@@ -870,10 +870,10 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>100</v>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>347749</v>
+        <v>347738</v>
       </c>
     </row>
     <row r="3">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6">

</xml_diff>